<commit_message>
Update Crop residues file
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/Crop residues.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/Crop residues.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A886EF9F-F338-4EF3-912C-2738641509DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55935444-07CC-413C-846B-EAF2D2B1CD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-980" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -2012,7 +2012,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2085,6 +2085,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -2129,7 +2136,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2171,6 +2178,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2563,38 +2571,38 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A2:O26"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" customWidth="1"/>
-    <col min="2" max="2" width="52.08984375" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="52.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>624</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>648</v>
       </c>
@@ -2603,7 +2611,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>625</v>
       </c>
@@ -2614,7 +2622,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>627</v>
       </c>
@@ -2625,7 +2633,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>628</v>
       </c>
@@ -2636,7 +2644,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>384</v>
       </c>
@@ -2650,7 +2658,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>626</v>
       </c>
@@ -2664,7 +2672,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>632</v>
       </c>
@@ -2675,7 +2683,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>112</v>
       </c>
@@ -2686,7 +2694,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>110</v>
       </c>
@@ -2694,7 +2702,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>108</v>
       </c>
@@ -2702,12 +2710,12 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>649</v>
       </c>
@@ -2715,7 +2723,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>642</v>
       </c>
@@ -2723,7 +2731,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>652</v>
       </c>
@@ -2741,13 +2749,13 @@
     <tabColor theme="2" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A2:H115"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="32.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>638</v>
       </c>
@@ -2755,7 +2763,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="111.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="111.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -2777,7 +2785,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>1</v>
       </c>
@@ -2803,7 +2811,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -2829,7 +2837,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -2855,7 +2863,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -2881,7 +2889,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -2907,7 +2915,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -2933,7 +2941,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2959,7 +2967,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2985,7 +2993,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -3011,7 +3019,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -3037,7 +3045,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -3063,7 +3071,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -3089,7 +3097,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -3115,7 +3123,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -3141,7 +3149,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -3167,7 +3175,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -3193,7 +3201,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -3219,7 +3227,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -3245,7 +3253,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -3271,7 +3279,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -3297,7 +3305,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -3323,7 +3331,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -3349,7 +3357,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -3375,7 +3383,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -3401,7 +3409,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -3427,7 +3435,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -3453,7 +3461,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -3479,7 +3487,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -3505,7 +3513,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -3531,7 +3539,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -3557,7 +3565,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -3583,7 +3591,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -3609,7 +3617,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -3635,7 +3643,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -3661,7 +3669,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -3687,7 +3695,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -3713,7 +3721,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -3739,7 +3747,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -3765,7 +3773,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -3791,7 +3799,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -3817,7 +3825,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -3843,7 +3851,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -3869,7 +3877,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -3895,7 +3903,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -3921,7 +3929,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -3947,7 +3955,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -3973,7 +3981,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -3999,7 +4007,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -4025,7 +4033,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -4051,7 +4059,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -4077,7 +4085,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -4103,7 +4111,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -4129,7 +4137,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -4155,7 +4163,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -4181,7 +4189,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -4207,7 +4215,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
@@ -4233,7 +4241,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
@@ -4259,7 +4267,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
@@ -4285,7 +4293,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -4311,7 +4319,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
@@ -4337,7 +4345,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
@@ -4363,7 +4371,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>64</v>
       </c>
@@ -4389,7 +4397,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
@@ -4415,7 +4423,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
@@ -4441,7 +4449,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
@@ -4467,7 +4475,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
@@ -4493,7 +4501,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
@@ -4519,7 +4527,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
@@ -4545,7 +4553,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
@@ -4571,7 +4579,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
@@ -4597,7 +4605,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
@@ -4623,7 +4631,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
@@ -4649,7 +4657,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
@@ -4675,7 +4683,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
@@ -4701,7 +4709,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
@@ -4727,7 +4735,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -4753,7 +4761,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>79</v>
       </c>
@@ -4779,7 +4787,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
@@ -4805,7 +4813,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>81</v>
       </c>
@@ -4831,7 +4839,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>82</v>
       </c>
@@ -4857,7 +4865,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>83</v>
       </c>
@@ -4883,7 +4891,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>84</v>
       </c>
@@ -4909,7 +4917,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>85</v>
       </c>
@@ -4935,7 +4943,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>86</v>
       </c>
@@ -4961,7 +4969,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>87</v>
       </c>
@@ -4987,7 +4995,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>88</v>
       </c>
@@ -5013,7 +5021,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>89</v>
       </c>
@@ -5039,7 +5047,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>90</v>
       </c>
@@ -5065,7 +5073,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>91</v>
       </c>
@@ -5091,7 +5099,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>92</v>
       </c>
@@ -5117,7 +5125,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>93</v>
       </c>
@@ -5143,7 +5151,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>94</v>
       </c>
@@ -5169,7 +5177,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>95</v>
       </c>
@@ -5195,7 +5203,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>96</v>
       </c>
@@ -5221,7 +5229,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>97</v>
       </c>
@@ -5247,7 +5255,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>98</v>
       </c>
@@ -5273,7 +5281,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>99</v>
       </c>
@@ -5299,7 +5307,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>100</v>
       </c>
@@ -5325,7 +5333,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>101</v>
       </c>
@@ -5351,7 +5359,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>102</v>
       </c>
@@ -5377,7 +5385,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>103</v>
       </c>
@@ -5403,7 +5411,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>104</v>
       </c>
@@ -5413,23 +5421,24 @@
       <c r="C106" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D106" s="6">
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="E106" s="6">
+      <c r="D106" s="4">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="E106" s="4">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="F106" s="6">
-        <v>1</v>
-      </c>
-      <c r="G106" s="6">
-        <v>0.22</v>
-      </c>
-      <c r="H106" s="6">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F106" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="G106" s="23">
+        <f>AVERAGE(G107:G108)</f>
+        <v>0.255</v>
+      </c>
+      <c r="H106" s="4">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>105</v>
       </c>
@@ -5455,7 +5464,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>106</v>
       </c>
@@ -5481,37 +5490,37 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -5528,20 +5537,20 @@
     <tabColor theme="2" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A2:GT115"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="32.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="8.54296875" style="1" customWidth="1"/>
-    <col min="5" max="202" width="5.6328125" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" style="1" customWidth="1"/>
+    <col min="5" max="202" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:202" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:202" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:202" ht="78.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -6142,7 +6151,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="5" spans="1:202" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:202" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>1</v>
       </c>
@@ -6750,7 +6759,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="6" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -6765,7 +6774,7 @@
       </c>
       <c r="FT6" s="1"/>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -6780,7 +6789,7 @@
       </c>
       <c r="FT7" s="1"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -6797,7 +6806,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -6812,7 +6821,7 @@
       </c>
       <c r="FT9" s="1"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -6827,7 +6836,7 @@
       </c>
       <c r="FT10" s="1"/>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -6844,7 +6853,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -6859,7 +6868,7 @@
       </c>
       <c r="FT12" s="16"/>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -6874,7 +6883,7 @@
       </c>
       <c r="FT13" s="1"/>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -6891,7 +6900,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -6908,7 +6917,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:202" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -6925,7 +6934,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -6942,7 +6951,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -6957,7 +6966,7 @@
       </c>
       <c r="FT18" s="16"/>
     </row>
-    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -6972,7 +6981,7 @@
       </c>
       <c r="FT19" s="1"/>
     </row>
-    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -6989,7 +6998,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -7004,7 +7013,7 @@
       </c>
       <c r="FT21" s="16"/>
     </row>
-    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -7021,7 +7030,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -7036,7 +7045,7 @@
       </c>
       <c r="FT23" s="1"/>
     </row>
-    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -7053,7 +7062,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -7068,7 +7077,7 @@
       </c>
       <c r="FT25" s="1"/>
     </row>
-    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -7085,7 +7094,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -7100,7 +7109,7 @@
       </c>
       <c r="FT27" s="1"/>
     </row>
-    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -7118,7 +7127,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -7135,7 +7144,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -7151,7 +7160,7 @@
       <c r="M30" s="6"/>
       <c r="FT30" s="16"/>
     </row>
-    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -7166,7 +7175,7 @@
       </c>
       <c r="FT31" s="16"/>
     </row>
-    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -7181,7 +7190,7 @@
       </c>
       <c r="FT32" s="1"/>
     </row>
-    <row r="33" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -7196,7 +7205,7 @@
       </c>
       <c r="FT33" s="1"/>
     </row>
-    <row r="34" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -7211,7 +7220,7 @@
       </c>
       <c r="FT34" s="1"/>
     </row>
-    <row r="35" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -7226,7 +7235,7 @@
       </c>
       <c r="FT35" s="1"/>
     </row>
-    <row r="36" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -7241,7 +7250,7 @@
       </c>
       <c r="FT36" s="1"/>
     </row>
-    <row r="37" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -7258,7 +7267,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -7275,7 +7284,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -7292,7 +7301,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -7307,7 +7316,7 @@
       </c>
       <c r="FT40" s="16"/>
     </row>
-    <row r="41" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -7322,7 +7331,7 @@
       </c>
       <c r="FT41" s="16"/>
     </row>
-    <row r="42" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -7337,7 +7346,7 @@
       </c>
       <c r="FT42" s="16"/>
     </row>
-    <row r="43" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -7352,7 +7361,7 @@
       </c>
       <c r="FT43" s="16"/>
     </row>
-    <row r="44" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -7367,7 +7376,7 @@
       </c>
       <c r="FT44" s="19"/>
     </row>
-    <row r="45" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -7384,7 +7393,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -7399,7 +7408,7 @@
       </c>
       <c r="FT46" s="16"/>
     </row>
-    <row r="47" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -7416,7 +7425,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="48" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -7431,7 +7440,7 @@
       </c>
       <c r="FT48" s="19"/>
     </row>
-    <row r="49" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -7446,7 +7455,7 @@
       </c>
       <c r="FT49" s="19"/>
     </row>
-    <row r="50" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -7461,7 +7470,7 @@
       </c>
       <c r="FT50" s="19"/>
     </row>
-    <row r="51" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -7478,7 +7487,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="52" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -7493,7 +7502,7 @@
       </c>
       <c r="FT52" s="19"/>
     </row>
-    <row r="53" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -7510,7 +7519,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -7527,7 +7536,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -7544,7 +7553,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -7559,7 +7568,7 @@
       </c>
       <c r="FT56" s="16"/>
     </row>
-    <row r="57" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -7576,7 +7585,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -7591,7 +7600,7 @@
       </c>
       <c r="FT58" s="16"/>
     </row>
-    <row r="59" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -7606,7 +7615,7 @@
       </c>
       <c r="FT59" s="16"/>
     </row>
-    <row r="60" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
@@ -7623,7 +7632,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="61" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
@@ -7638,7 +7647,7 @@
       </c>
       <c r="FT61" s="1"/>
     </row>
-    <row r="62" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
@@ -7653,7 +7662,7 @@
       </c>
       <c r="FT62" s="1"/>
     </row>
-    <row r="63" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -7670,7 +7679,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="64" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
@@ -7685,7 +7694,7 @@
       </c>
       <c r="FT64" s="1"/>
     </row>
-    <row r="65" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
@@ -7702,7 +7711,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>64</v>
       </c>
@@ -7717,7 +7726,7 @@
       </c>
       <c r="FT66" s="1"/>
     </row>
-    <row r="67" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
@@ -7732,7 +7741,7 @@
       </c>
       <c r="FT67" s="1"/>
     </row>
-    <row r="68" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
@@ -7749,7 +7758,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
@@ -7764,7 +7773,7 @@
       </c>
       <c r="FT69" s="1"/>
     </row>
-    <row r="70" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
@@ -7781,7 +7790,7 @@
         <v>0.14333333333333334</v>
       </c>
     </row>
-    <row r="71" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
@@ -7796,7 +7805,7 @@
       </c>
       <c r="FT71" s="1"/>
     </row>
-    <row r="72" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
@@ -7811,7 +7820,7 @@
       </c>
       <c r="FT72" s="1"/>
     </row>
-    <row r="73" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
@@ -7828,7 +7837,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
@@ -7845,7 +7854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
@@ -7862,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
@@ -7877,7 +7886,7 @@
       </c>
       <c r="FT76" s="1"/>
     </row>
-    <row r="77" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
@@ -7894,7 +7903,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="78" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
@@ -7909,7 +7918,7 @@
       </c>
       <c r="FT78" s="1"/>
     </row>
-    <row r="79" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
@@ -7924,7 +7933,7 @@
       </c>
       <c r="FT79" s="1"/>
     </row>
-    <row r="80" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -7941,7 +7950,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>79</v>
       </c>
@@ -7958,7 +7967,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="82" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
@@ -7973,7 +7982,7 @@
       </c>
       <c r="FT82" s="1"/>
     </row>
-    <row r="83" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>81</v>
       </c>
@@ -7988,7 +7997,7 @@
       </c>
       <c r="FT83" s="1"/>
     </row>
-    <row r="84" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>82</v>
       </c>
@@ -8005,7 +8014,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>83</v>
       </c>
@@ -8022,7 +8031,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>84</v>
       </c>
@@ -8039,7 +8048,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>85</v>
       </c>
@@ -8056,7 +8065,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="88" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>86</v>
       </c>
@@ -8071,7 +8080,7 @@
       </c>
       <c r="FT88" s="1"/>
     </row>
-    <row r="89" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>87</v>
       </c>
@@ -8088,7 +8097,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="90" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>88</v>
       </c>
@@ -8103,7 +8112,7 @@
       </c>
       <c r="FT90" s="1"/>
     </row>
-    <row r="91" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>89</v>
       </c>
@@ -8120,7 +8129,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="92" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>90</v>
       </c>
@@ -8135,7 +8144,7 @@
       </c>
       <c r="FT92" s="1"/>
     </row>
-    <row r="93" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>91</v>
       </c>
@@ -8152,7 +8161,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="94" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>92</v>
       </c>
@@ -8169,7 +8178,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="95" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>93</v>
       </c>
@@ -8186,7 +8195,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>94</v>
       </c>
@@ -8201,7 +8210,7 @@
       </c>
       <c r="FT96" s="1"/>
     </row>
-    <row r="97" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>95</v>
       </c>
@@ -8216,7 +8225,7 @@
       </c>
       <c r="FT97" s="1"/>
     </row>
-    <row r="98" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>96</v>
       </c>
@@ -8231,7 +8240,7 @@
       </c>
       <c r="FT98" s="1"/>
     </row>
-    <row r="99" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>97</v>
       </c>
@@ -8246,7 +8255,7 @@
       </c>
       <c r="FT99" s="1"/>
     </row>
-    <row r="100" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>98</v>
       </c>
@@ -8263,7 +8272,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="101" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>99</v>
       </c>
@@ -8278,7 +8287,7 @@
       </c>
       <c r="FT101" s="17"/>
     </row>
-    <row r="102" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>100</v>
       </c>
@@ -8295,7 +8304,7 @@
         <v>0.14299999999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>101</v>
       </c>
@@ -8310,7 +8319,7 @@
       </c>
       <c r="FT103" s="1"/>
     </row>
-    <row r="104" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>102</v>
       </c>
@@ -8325,7 +8334,7 @@
       </c>
       <c r="FT104" s="1"/>
     </row>
-    <row r="105" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>103</v>
       </c>
@@ -8340,7 +8349,7 @@
       </c>
       <c r="FT105" s="1"/>
     </row>
-    <row r="106" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>104</v>
       </c>
@@ -8357,7 +8366,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>105</v>
       </c>
@@ -8374,7 +8383,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="108" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>106</v>
       </c>
@@ -8391,37 +8400,37 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="109" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:176" x14ac:dyDescent="0.3">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -8433,23 +8442,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100A603BB68AE5C0F4C908E70EB4D1DDDC3" ma:contentTypeVersion="15" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="bc1901b771652496ef02f4cbdf878f9e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95" xmlns:ns4="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c61e44642a1e9e2aad865b2f0b39e8f" ns3:_="" ns4:_="">
     <xsd:import namespace="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95"/>
@@ -8684,25 +8676,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27BF0A1B-B2BC-4159-BD4C-213AA0853490}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8719,4 +8710,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>